<commit_message>
docs: simplify required AWS deployment inputs
</commit_message>
<xml_diff>
--- a/docs/operation/aws-resource-parameter-sheet.xlsx
+++ b/docs/operation/aws-resource-parameter-sheet.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使い方・前提" sheetId="1" r:id="Ra23353f691ea42e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_AWSリソース一覧" sheetId="2" r:id="R51766eb347d748c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Terraform入力値" sheetId="3" r:id="Rc919bf1f557b40d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ファイル編集マップ" sheetId="4" r:id="R69e1aac72bda4226"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Terraform出力・取得値" sheetId="5" r:id="R5bfdc53f460d4a72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Deploy環境変数" sheetId="6" r:id="R9536390e3084478e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_コスト・保持期間" sheetId="7" r:id="Rdf11ed0c693340ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Category-C検証" sheetId="8" r:id="R6581f0ca69c34af0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_destroy前確認" sheetId="9" r:id="R3ef9fb92eb5941c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使い方・前提" sheetId="1" r:id="Rf881e057e72a4682"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_AWSリソース一覧" sheetId="2" r:id="R35ed67d5e0b64b20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Terraform入力値" sheetId="3" r:id="Rcb81db667f1f4eb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ファイル編集マップ" sheetId="4" r:id="R4a098e186852453f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Terraform出力・取得値" sheetId="5" r:id="R53971994e14d4014"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Deploy環境変数" sheetId="6" r:id="Reb6a32220960460d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_コスト・保持期間" sheetId="7" r:id="R873d9ae7e7254ef7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Category-C検証" sheetId="8" r:id="R1c2bcc54ca484a16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_destroy前確認" sheetId="9" r:id="R71c881ba90f2482b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="6">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -55,8 +55,32 @@
       <x:color rgb="FF222222"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF595959"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF7F6000"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -73,8 +97,38 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDEBF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDEBF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="8">
+  <x:borders count="16">
     <x:border/>
     <x:border>
       <x:right style="thin">
@@ -132,11 +186,90 @@
         <x:color rgb="FFFFFFFF"/>
       </x:right>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD6B656"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD6B656"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD6B656"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD6B656"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD6B656"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD6B656"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="37">
+  <x:cellXfs count="91">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -253,10 +386,162 @@
         </x:ext>
       </x:extLst>
     </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
+  <x:dxfs count="2">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+  </x:dxfs>
 </x:styleSheet>
 </file>
 
@@ -305,7 +590,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TerraformInputTable" displayName="TerraformInputTable" ref="A4:S284" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TerraformInputTable" displayName="TerraformInputTable" ref="A4:S285" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="19">
     <x:tableColumn id="1" name="AWSサービス/領域"/>
     <x:tableColumn id="2" name="リソース/用途"/>
@@ -621,8 +906,14 @@
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="110" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="7" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="46" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="43" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="50" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="35" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
@@ -673,7 +964,7 @@
         <x:v>入力色</x:v>
       </x:c>
       <x:c r="B8" s="25" t="str">
-        <x:v>黄色は環境固有値への置換・確認が必要な項目。実値はSSM/Secrets Managerまたは実行時環境変数で供給する。</x:v>
+        <x:v>作業者が直接確認するのは下表12項目。01〜08シートは参照台帳であり、全行レビューや既定値の転記は不要。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -724,10 +1015,389 @@
         <x:v>docs/operation/aws-build-procedure.md</x:v>
       </x:c>
     </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="37"/>
+      <x:c r="B16" s="37" t="str">
+        <x:v>構築前の必須確認</x:v>
+      </x:c>
+      <x:c r="C16" s="37"/>
+      <x:c r="D16" s="37"/>
+      <x:c r="E16" s="37"/>
+      <x:c r="F16" s="37"/>
+      <x:c r="G16" s="37"/>
+      <x:c r="H16" s="37"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="39"/>
+      <x:c r="B17" s="39" t="str">
+        <x:v>通常のdev構築で人が判断・入力する項目は次の12件だけです。記録列には実ARN、アカウントID、ドメイン、メール、Secretを書かないでください。</x:v>
+      </x:c>
+      <x:c r="C17" s="39"/>
+      <x:c r="D17" s="39"/>
+      <x:c r="E17" s="39"/>
+      <x:c r="F17" s="39"/>
+      <x:c r="G17" s="39"/>
+      <x:c r="H17" s="39"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="82" t="str">
+        <x:v>未完了件数</x:v>
+      </x:c>
+      <x:c r="B18" s="83" t="n">
+        <x:f>COUNTIF(G21:G32,"&lt;&gt;確認済み")</x:f>
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="32" customHeight="1">
+      <x:c r="A20" s="84" t="str">
+        <x:v>No.</x:v>
+      </x:c>
+      <x:c r="B20" s="84" t="str">
+        <x:v>確認対象</x:v>
+      </x:c>
+      <x:c r="C20" s="84" t="str">
+        <x:v>実施手順</x:v>
+      </x:c>
+      <x:c r="D20" s="84" t="str">
+        <x:v>合格条件</x:v>
+      </x:c>
+      <x:c r="E20" s="84" t="str">
+        <x:v>実値の設定先</x:v>
+      </x:c>
+      <x:c r="F20" s="84" t="str">
+        <x:v>作業区分</x:v>
+      </x:c>
+      <x:c r="G20" s="84" t="str">
+        <x:v>状態</x:v>
+      </x:c>
+      <x:c r="H20" s="84" t="str">
+        <x:v>記録（実値を書かない）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="48" customHeight="1">
+      <x:c r="A21" s="76" t="str">
+        <x:v>01</x:v>
+      </x:c>
+      <x:c r="B21" s="77" t="str">
+        <x:v>AWSアカウント・実行role・リージョン</x:v>
+      </x:c>
+      <x:c r="C21" s="77" t="str">
+        <x:v>BP-01</x:v>
+      </x:c>
+      <x:c r="D21" s="63" t="str">
+        <x:v>検証用アカウント、root以外、ap-northeast-1</x:v>
+      </x:c>
+      <x:c r="E21" s="63" t="str">
+        <x:v>AWS profile/session、作業記録</x:v>
+      </x:c>
+      <x:c r="F21" s="87" t="str">
+        <x:v>確認</x:v>
+      </x:c>
+      <x:c r="G21" s="89" t="str">
+        <x:v>未確認</x:v>
+      </x:c>
+      <x:c r="H21" s="64" t="str">
+        <x:v>Account IDやARNは記載しない</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="48" customHeight="1">
+      <x:c r="A22" s="78" t="str">
+        <x:v>02</x:v>
+      </x:c>
+      <x:c r="B22" s="79" t="str">
+        <x:v>予算アラート・停止判断者</x:v>
+      </x:c>
+      <x:c r="C22" s="79" t="str">
+        <x:v>BP-01</x:v>
+      </x:c>
+      <x:c r="D22" s="66" t="str">
+        <x:v>予算アラート有効、停止判断者が確定</x:v>
+      </x:c>
+      <x:c r="E22" s="66" t="str">
+        <x:v>AWS Budgets、作業記録</x:v>
+      </x:c>
+      <x:c r="F22" s="88" t="str">
+        <x:v>確認</x:v>
+      </x:c>
+      <x:c r="G22" s="90" t="str">
+        <x:v>未確認</x:v>
+      </x:c>
+      <x:c r="H22" s="67" t="str">
+        <x:v>設定済みと担当者だけを記録</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="48" customHeight="1">
+      <x:c r="A23" s="78" t="str">
+        <x:v>03</x:v>
+      </x:c>
+      <x:c r="B23" s="79" t="str">
+        <x:v>ALB用ACM証明書</x:v>
+      </x:c>
+      <x:c r="C23" s="79" t="str">
+        <x:v>BP-02/BP-05</x:v>
+      </x:c>
+      <x:c r="D23" s="66" t="str">
+        <x:v>ap-northeast-1、対象domain、ISSUED</x:v>
+      </x:c>
+      <x:c r="E23" s="66" t="str">
+        <x:v>SSM /ops-platform/dev/alb-certificate-arn</x:v>
+      </x:c>
+      <x:c r="F23" s="88" t="str">
+        <x:v>入力</x:v>
+      </x:c>
+      <x:c r="G23" s="90" t="str">
+        <x:v>未確認</x:v>
+      </x:c>
+      <x:c r="H23" s="67" t="str">
+        <x:v>SSM登録済みとだけ記録</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="48" customHeight="1">
+      <x:c r="A24" s="78" t="str">
+        <x:v>04</x:v>
+      </x:c>
+      <x:c r="B24" s="79" t="str">
+        <x:v>CodeStar Connection</x:v>
+      </x:c>
+      <x:c r="C24" s="79" t="str">
+        <x:v>BP-02</x:v>
+      </x:c>
+      <x:c r="D24" s="66" t="str">
+        <x:v>GitHub接続がAVAILABLE</x:v>
+      </x:c>
+      <x:c r="E24" s="66" t="str">
+        <x:v>bootstrap/terraform.tfvars</x:v>
+      </x:c>
+      <x:c r="F24" s="88" t="str">
+        <x:v>入力</x:v>
+      </x:c>
+      <x:c r="G24" s="90" t="str">
+        <x:v>未確認</x:v>
+      </x:c>
+      <x:c r="H24" s="67" t="str">
+        <x:v>terraform.tfvars設定済みとだけ記録</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="48" customHeight="1">
+      <x:c r="A25" s="78" t="str">
+        <x:v>05</x:v>
+      </x:c>
+      <x:c r="B25" s="79" t="str">
+        <x:v>Source repository / branch</x:v>
+      </x:c>
+      <x:c r="C25" s="79" t="str">
+        <x:v>BP-02</x:v>
+      </x:c>
+      <x:c r="D25" s="66" t="str">
+        <x:v>owner/repositoryが正しく、branchはmain</x:v>
+      </x:c>
+      <x:c r="E25" s="66" t="str">
+        <x:v>bootstrap/terraform.tfvars</x:v>
+      </x:c>
+      <x:c r="F25" s="88" t="str">
+        <x:v>入力</x:v>
+      </x:c>
+      <x:c r="G25" s="90" t="str">
+        <x:v>未確認</x:v>
+      </x:c>
+      <x:c r="H25" s="67" t="str">
+        <x:v>設定済みとだけ記録</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="48" customHeight="1">
+      <x:c r="A26" s="78" t="str">
+        <x:v>06</x:v>
+      </x:c>
+      <x:c r="B26" s="79" t="str">
+        <x:v>ALB HTTPS許可CIDR</x:v>
+      </x:c>
+      <x:c r="C26" s="79" t="str">
+        <x:v>BP-05</x:v>
+      </x:c>
+      <x:c r="D26" s="66" t="str">
+        <x:v>承認済みJSON配列、0.0.0.0/0を含まない</x:v>
+      </x:c>
+      <x:c r="E26" s="66" t="str">
+        <x:v>SSM /ops-platform/dev/alb-ingress-cidrs</x:v>
+      </x:c>
+      <x:c r="F26" s="88" t="str">
+        <x:v>入力</x:v>
+      </x:c>
+      <x:c r="G26" s="90" t="str">
+        <x:v>未確認</x:v>
+      </x:c>
+      <x:c r="H26" s="67" t="str">
+        <x:v>SSM登録済みとだけ記録</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="48" customHeight="1">
+      <x:c r="A27" s="78" t="str">
+        <x:v>07</x:v>
+      </x:c>
+      <x:c r="B27" s="79" t="str">
+        <x:v>EKS API許可CIDR</x:v>
+      </x:c>
+      <x:c r="C27" s="79" t="str">
+        <x:v>BP-05</x:v>
+      </x:c>
+      <x:c r="D27" s="66" t="str">
+        <x:v>kubectl接続元のJSON配列、0.0.0.0/0を含まない</x:v>
+      </x:c>
+      <x:c r="E27" s="66" t="str">
+        <x:v>SSM /ops-platform/dev/eks-public-access-cidrs</x:v>
+      </x:c>
+      <x:c r="F27" s="88" t="str">
+        <x:v>入力</x:v>
+      </x:c>
+      <x:c r="G27" s="90" t="str">
+        <x:v>未確認</x:v>
+      </x:c>
+      <x:c r="H27" s="67" t="str">
+        <x:v>SSM登録済みとだけ記録</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="48" customHeight="1">
+      <x:c r="A28" s="78" t="str">
+        <x:v>08</x:v>
+      </x:c>
+      <x:c r="B28" s="79" t="str">
+        <x:v>EKS Operator role</x:v>
+      </x:c>
+      <x:c r="C28" s="79" t="str">
+        <x:v>BP-05</x:v>
+      </x:c>
+      <x:c r="D28" s="66" t="str">
+        <x:v>承認済みIAM role ARN</x:v>
+      </x:c>
+      <x:c r="E28" s="66" t="str">
+        <x:v>SSM /ops-platform/dev/eks-operator-principal-arn</x:v>
+      </x:c>
+      <x:c r="F28" s="88" t="str">
+        <x:v>入力</x:v>
+      </x:c>
+      <x:c r="G28" s="90" t="str">
+        <x:v>未確認</x:v>
+      </x:c>
+      <x:c r="H28" s="67" t="str">
+        <x:v>SSM登録済みとだけ記録</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="48" customHeight="1">
+      <x:c r="A29" s="78" t="str">
+        <x:v>09</x:v>
+      </x:c>
+      <x:c r="B29" s="79" t="str">
+        <x:v>Migration起動主体</x:v>
+      </x:c>
+      <x:c r="C29" s="79" t="str">
+        <x:v>BP-05</x:v>
+      </x:c>
+      <x:c r="D29" s="66" t="str">
+        <x:v>承認済みrole ARNのJSON配列</x:v>
+      </x:c>
+      <x:c r="E29" s="66" t="str">
+        <x:v>SSM /ops-platform/dev/migration-launcher-principal-arns</x:v>
+      </x:c>
+      <x:c r="F29" s="88" t="str">
+        <x:v>入力</x:v>
+      </x:c>
+      <x:c r="G29" s="90" t="str">
+        <x:v>未確認</x:v>
+      </x:c>
+      <x:c r="H29" s="67" t="str">
+        <x:v>SSM登録済みとだけ記録</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="48" customHeight="1">
+      <x:c r="A30" s="78" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B30" s="79" t="str">
+        <x:v>初回起動ゲート</x:v>
+      </x:c>
+      <x:c r="C30" s="79" t="str">
+        <x:v>BP-05</x:v>
+      </x:c>
+      <x:c r="D30" s="66" t="str">
+        <x:v>ecs_desired_count=0、SNS subscription=false</x:v>
+      </x:c>
+      <x:c r="E30" s="66" t="str">
+        <x:v>SSMの2パラメータ</x:v>
+      </x:c>
+      <x:c r="F30" s="88" t="str">
+        <x:v>入力</x:v>
+      </x:c>
+      <x:c r="G30" s="90" t="str">
+        <x:v>未確認</x:v>
+      </x:c>
+      <x:c r="H30" s="67" t="str">
+        <x:v>両パラメータのversionだけを記録</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="48" customHeight="1">
+      <x:c r="A31" s="78" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B31" s="79" t="str">
+        <x:v>コスト・保持・destroy方針</x:v>
+      </x:c>
+      <x:c r="C31" s="79" t="str">
+        <x:v>BP-07前</x:v>
+      </x:c>
+      <x:c r="D31" s="66" t="str">
+        <x:v>NAT/Aurora/EKS/WAF等とsnapshot責任者を承認</x:v>
+      </x:c>
+      <x:c r="E31" s="66" t="str">
+        <x:v>作業記録。詳細は06/08シート</x:v>
+      </x:c>
+      <x:c r="F31" s="88" t="str">
+        <x:v>確認</x:v>
+      </x:c>
+      <x:c r="G31" s="90" t="str">
+        <x:v>未確認</x:v>
+      </x:c>
+      <x:c r="H31" s="67" t="str">
+        <x:v>判断結果と担当者だけを記録</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="48" customHeight="1">
+      <x:c r="A32" s="78" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B32" s="79" t="str">
+        <x:v>EKS versionのサポート状態</x:v>
+      </x:c>
+      <x:c r="C32" s="79" t="str">
+        <x:v>BP-07直前</x:v>
+      </x:c>
+      <x:c r="D32" s="66" t="str">
+        <x:v>apply時点でStandard Support対象</x:v>
+      </x:c>
+      <x:c r="E32" s="66" t="str">
+        <x:v>AWS公式情報、infra/environments/dev/variables.tf</x:v>
+      </x:c>
+      <x:c r="F32" s="88" t="str">
+        <x:v>確認</x:v>
+      </x:c>
+      <x:c r="G32" s="90" t="str">
+        <x:v>未確認</x:v>
+      </x:c>
+      <x:c r="H32" s="67" t="str">
+        <x:v>確認日とversionだけを記録</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
+  <x:conditionalFormatting sqref="G21:G32">
+    <x:cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="確認済み"/>
+  </x:conditionalFormatting>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="G21:G32">
+      <x:formula1>"未確認,確認済み"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d1d26ed59674f3a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c3ec9f68a9b4b97"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7231,7 +7901,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd41c1a972cd54eb9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb285f8f4608147ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7271,7 +7941,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>全variableから抽出。280項目。黄色列は環境固有値を確認する。</x:v>
+        <x:v>全variableの参照台帳。作業者が全280項目を確認する必要はなく、先頭シートの必須12項目だけを使用する。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="30" customHeight="1"/>
@@ -14027,28 +14697,28 @@
         <x:v>list(string)</x:v>
       </x:c>
       <x:c r="I118" s="22" t="str">
-        <x:v>任意（既定値あり）</x:v>
+        <x:v>必須</x:v>
       </x:c>
       <x:c r="J118" s="22" t="str">
-        <x:v>["203.0.113.0/24"]（詳細は対象ファイル参照）</x:v>
+        <x:v>なし</x:v>
       </x:c>
       <x:c r="K118" s="22" t="str">
-        <x:v>["203.0.113.0/24"]（詳細は対象ファイル参照）</x:v>
+        <x:v>承認済み接続元CIDRのJSON配列</x:v>
       </x:c>
       <x:c r="L118" s="24" t="str">
-        <x:v>必要時</x:v>
+        <x:v>必要</x:v>
       </x:c>
       <x:c r="M118" s="24" t="str">
-        <x:v>variables.tf既定値または承認済みPipeline入力</x:v>
+        <x:v>SSM Parameter Store</x:v>
       </x:c>
       <x:c r="N118" s="24" t="str">
-        <x:v>variables.tf既定値または承認済みPipeline入力</x:v>
+        <x:v>/ops-platform/dev/alb-ingress-cidrs</x:v>
       </x:c>
       <x:c r="O118" s="24" t="str">
         <x:v>非機微</x:v>
       </x:c>
       <x:c r="P118" s="22" t="str">
-        <x:v>未設定時: 既定値を使用</x:v>
+        <x:v>未設定時: Pipeline plan不能</x:v>
       </x:c>
       <x:c r="Q118" s="22" t="str">
         <x:v>小/間接的</x:v>
@@ -14057,7 +14727,7 @@
         <x:v>plan出力とAWS Console/CLIで確認</x:v>
       </x:c>
       <x:c r="S118" s="23" t="str">
-        <x:v>7</x:v>
+        <x:v>3,5,7</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="30" customHeight="1">
@@ -23854,10 +24524,69 @@
         <x:v>7</x:v>
       </x:c>
     </x:row>
+    <x:row r="285">
+      <x:c r="A285" t="str">
+        <x:v>PIPELINE</x:v>
+      </x:c>
+      <x:c r="B285" t="str">
+        <x:v>pipeline_alb_ingress_cidrs_parameter_name</x:v>
+      </x:c>
+      <x:c r="C285" t="str">
+        <x:v>bootstrap</x:v>
+      </x:c>
+      <x:c r="D285" t="str">
+        <x:v>variable.pipeline_alb_ingress_cidrs_parameter_name</x:v>
+      </x:c>
+      <x:c r="E285" t="str">
+        <x:v>pipeline_alb_ingress_cidrs_parameter_name</x:v>
+      </x:c>
+      <x:c r="F285" t="str">
+        <x:v>bootstrap/variables.tf</x:v>
+      </x:c>
+      <x:c r="G285" t="str">
+        <x:v>variable "pipeline_alb_ingress_cidrs_parameter_name"</x:v>
+      </x:c>
+      <x:c r="H285" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="I285" t="str">
+        <x:v>任意（既定値あり）</x:v>
+      </x:c>
+      <x:c r="J285" t="str">
+        <x:v>/ops-platform/dev/alb-ingress-cidrs</x:v>
+      </x:c>
+      <x:c r="K285" t="str">
+        <x:v>/ops-platform/dev/alb-ingress-cidrs</x:v>
+      </x:c>
+      <x:c r="L285" t="str">
+        <x:v>不要（既定値使用）</x:v>
+      </x:c>
+      <x:c r="M285" t="str">
+        <x:v>variables.tf既定値</x:v>
+      </x:c>
+      <x:c r="N285" t="str">
+        <x:v>CodeBuild環境変数経由</x:v>
+      </x:c>
+      <x:c r="O285" t="str">
+        <x:v>非機微</x:v>
+      </x:c>
+      <x:c r="P285" t="str">
+        <x:v>未設定時: 既定値を使用</x:v>
+      </x:c>
+      <x:c r="Q285" t="str">
+        <x:v>小/間接的</x:v>
+      </x:c>
+      <x:c r="R285" t="str">
+        <x:v>手順5のSSM名と一致確認</x:v>
+      </x:c>
+      <x:c r="S285" t="str">
+        <x:v>4-5</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R630d479ee0074db0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf5310d6d060456f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23885,7 +24614,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>手順通りに確認・供給する設定箇所。実値をリポジトリへ直接記載しない。</x:v>
+        <x:v>設定定義の参照先。対象ファイル名は直接編集の指示ではない。実作業は先頭シートと構築手順書に従う。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="30" customHeight="1"/>
@@ -23917,19 +24646,19 @@
         <x:v>事前入力</x:v>
       </x:c>
       <x:c r="B5" s="22" t="str">
-        <x:v>infra/environments/dev/variables.tf</x:v>
+        <x:v>SSM Parameter Store</x:v>
       </x:c>
       <x:c r="C5" s="22" t="str">
-        <x:v>alb_certificate_arn</x:v>
+        <x:v>/ops-platform/dev/alb-certificate-arn</x:v>
       </x:c>
       <x:c r="D5" s="22" t="str">
         <x:v>ACM証明書ARN</x:v>
       </x:c>
       <x:c r="E5" s="22" t="str">
-        <x:v>SSM Parameter Store</x:v>
+        <x:v>ACM describe-certificate</x:v>
       </x:c>
       <x:c r="F5" s="22" t="str">
-        <x:v>実ARNは記載しない</x:v>
+        <x:v>ISSUED・対象domain・ap-northeast-1</x:v>
       </x:c>
       <x:c r="G5" s="23" t="str">
         <x:v>2,5,7</x:v>
@@ -23940,19 +24669,19 @@
         <x:v>事前入力</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
-        <x:v>infra/environments/dev/variables.tf</x:v>
+        <x:v>SSM Parameter Store</x:v>
       </x:c>
       <x:c r="C6" s="22" t="str">
-        <x:v>eks_operator_principal_arn</x:v>
+        <x:v>/ops-platform/dev/eks-operator-principal-arn</x:v>
       </x:c>
       <x:c r="D6" s="22" t="str">
         <x:v>EKS管理主体ARN</x:v>
       </x:c>
       <x:c r="E6" s="22" t="str">
-        <x:v>SSM Parameter Store</x:v>
+        <x:v>組織IAM管理台帳</x:v>
       </x:c>
       <x:c r="F6" s="22" t="str">
-        <x:v>実ARNは記載しない</x:v>
+        <x:v>承認済みrole ARN</x:v>
       </x:c>
       <x:c r="G6" s="23" t="str">
         <x:v>2,5,7</x:v>
@@ -23963,19 +24692,19 @@
         <x:v>事前入力</x:v>
       </x:c>
       <x:c r="B7" s="22" t="str">
-        <x:v>infra/environments/dev/variables.tf</x:v>
+        <x:v>SSM Parameter Store</x:v>
       </x:c>
       <x:c r="C7" s="22" t="str">
-        <x:v>migration_launcher_trusted_principal_arns</x:v>
+        <x:v>/ops-platform/dev/migration-launcher-principal-arns</x:v>
       </x:c>
       <x:c r="D7" s="22" t="str">
         <x:v>migration起動主体</x:v>
       </x:c>
       <x:c r="E7" s="22" t="str">
-        <x:v>SSM Parameter Store(JSON配列)</x:v>
+        <x:v>組織IAM管理台帳</x:v>
       </x:c>
       <x:c r="F7" s="22" t="str">
-        <x:v>最低1主体</x:v>
+        <x:v>承認済みrole ARNのJSON配列</x:v>
       </x:c>
       <x:c r="G7" s="23" t="str">
         <x:v>2,5,7</x:v>
@@ -23986,22 +24715,22 @@
         <x:v>ネットワーク</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
-        <x:v>infra/environments/dev/variables.tf</x:v>
+        <x:v>SSM Parameter Store</x:v>
       </x:c>
       <x:c r="C8" s="22" t="str">
-        <x:v>network_*</x:v>
+        <x:v>alb-ingress-cidrs / eks-public-access-cidrs</x:v>
       </x:c>
       <x:c r="D8" s="22" t="str">
-        <x:v>VPC/AZ/subnet/CIDR</x:v>
+        <x:v>ALB/EKS接続元CIDR</x:v>
       </x:c>
       <x:c r="E8" s="22" t="str">
-        <x:v>Parameter Sheet承認値</x:v>
+        <x:v>接続元管理台帳</x:v>
       </x:c>
       <x:c r="F8" s="22" t="str">
-        <x:v>CIDR重複なし・ALB/EKSはworld-open禁止</x:v>
+        <x:v>JSON配列・0.0.0.0/0禁止</x:v>
       </x:c>
       <x:c r="G8" s="23" t="str">
-        <x:v>3,7</x:v>
+        <x:v>3,5,7</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -24306,7 +25035,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc985d46062e74913"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d340015dc294d07"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27982,7 +28711,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95d7f969905e4ab0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a3c3bc2a7d34313"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28396,7 +29125,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R233a0908fd02408c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0abc7daa936a445e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28707,7 +29436,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R775ec9a532094636"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82e503fb703e455d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29133,7 +29862,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc08d9ae848d84950"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28609e1cac8d43a6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29427,7 +30156,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6dd2ed5617aa4b76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ca855adf40b48e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>